<commit_message>
Renamed document and added our names in the excel
</commit_message>
<xml_diff>
--- a/Docs/Lab01/Lab01_ReviewReport.xlsx
+++ b/Docs/Lab01/Lab01_ReviewReport.xlsx
@@ -1,20 +1,36 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="Calc"/>
-  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
-  <workbookProtection/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+  <workbookPr defaultThemeVersion="202300"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\fac\sem6\VVSS-Lab\Docs\Lab01\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4AE20354-0E7B-4D3A-90F0-D4BC7611CD53}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" tabRatio="500" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Requirements Phase Defects" sheetId="1" state="visible" r:id="rId2"/>
-    <sheet name="Architect. Design Phase Defects" sheetId="2" state="visible" r:id="rId3"/>
-    <sheet name="Coding Phase Defects" sheetId="3" state="visible" r:id="rId4"/>
-    <sheet name="Tool-basedCodeAnalysis" sheetId="4" state="visible" r:id="rId5"/>
+    <sheet name="Requirements Phase Defects" sheetId="1" r:id="rId1"/>
+    <sheet name="Architect. Design Phase Defects" sheetId="2" r:id="rId2"/>
+    <sheet name="Coding Phase Defects" sheetId="3" r:id="rId3"/>
+    <sheet name="Tool-basedCodeAnalysis" sheetId="4" r:id="rId4"/>
   </sheets>
-  <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
+  <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="ExcelA1"/>
     </ext>
@@ -23,195 +39,195 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="88">
-  <si>
-    <t xml:space="preserve">do not print this form</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Echipa</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Review Form. Requirements Defects</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Numele si prenumele</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Grupa</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Student 1:</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hanza Casian</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Document  Title:</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Requirements Document</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Student 2:</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Goga Alexandru</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Author Name:</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Firicescu George</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Student 3:</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Iliuta Filip</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reviewer Name:</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="88">
+  <si>
+    <t>do not print this form</t>
+  </si>
+  <si>
+    <t>Echipa</t>
+  </si>
+  <si>
+    <t>Review Form. Requirements Defects</t>
+  </si>
+  <si>
+    <t>Numele si prenumele</t>
+  </si>
+  <si>
+    <t>Grupa</t>
+  </si>
+  <si>
+    <t>Student 1:</t>
+  </si>
+  <si>
+    <t>Hanza Casian</t>
+  </si>
+  <si>
+    <t>Document  Title:</t>
+  </si>
+  <si>
+    <t>Requirements Document</t>
+  </si>
+  <si>
+    <t>Student 2:</t>
+  </si>
+  <si>
+    <t>Goga Alexandru</t>
+  </si>
+  <si>
+    <t>Author Name:</t>
+  </si>
+  <si>
+    <t>Firicescu George</t>
+  </si>
+  <si>
+    <t>Student 3:</t>
+  </si>
+  <si>
+    <t>Iliuta Filip</t>
+  </si>
+  <si>
+    <t>Reviewer Name:</t>
   </si>
   <si>
     <t xml:space="preserve">Review date: </t>
   </si>
   <si>
-    <t xml:space="preserve">16.03.2025</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Crt. No.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Checked Item</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Doc. page/line</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Comments/ improvements</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R05</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F02a, F02b</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nu se specifica cum se face cautarea dupa nume (de exemplu daca cautam string-ul "produs", dorim produsele care incep astfel, sau cele care au numele strict "produs", sau cele care contin acest string?)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NU se ofera detalii despre ceea ce presupune gestiunea produselor si a pieselor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R07</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nu se precizeaza ce tip de aplicatie se doreste. (web, desktop, mobile etc)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Effort to review document (hours):</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Review Form. Architectural Design Defects</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Architectural Design Document</t>
+    <t>16.03.2025</t>
+  </si>
+  <si>
+    <t>Crt. No.</t>
+  </si>
+  <si>
+    <t>Checked Item</t>
+  </si>
+  <si>
+    <t>Doc. page/line</t>
+  </si>
+  <si>
+    <t>Comments/ improvements</t>
+  </si>
+  <si>
+    <t>R05</t>
+  </si>
+  <si>
+    <t>F02a, F02b</t>
+  </si>
+  <si>
+    <t>Nu se specifica cum se face cautarea dupa nume (de exemplu daca cautam string-ul "produs", dorim produsele care incep astfel, sau cele care au numele strict "produs", sau cele care contin acest string?)</t>
+  </si>
+  <si>
+    <t>R01</t>
+  </si>
+  <si>
+    <t>NU se ofera detalii despre ceea ce presupune gestiunea produselor si a pieselor</t>
+  </si>
+  <si>
+    <t>R07</t>
+  </si>
+  <si>
+    <t>Nu se precizeaza ce tip de aplicatie se doreste. (web, desktop, mobile etc)</t>
+  </si>
+  <si>
+    <t>Effort to review document (hours):</t>
+  </si>
+  <si>
+    <t>Review Form. Architectural Design Defects</t>
+  </si>
+  <si>
+    <t>Architectural Design Document</t>
   </si>
   <si>
     <t xml:space="preserve">Author Name: </t>
   </si>
   <si>
-    <t xml:space="preserve">Georgescu Anca</t>
-  </si>
-  <si>
-    <t xml:space="preserve">A05</t>
-  </si>
-  <si>
-    <t xml:space="preserve">In controller exista mesaje de eroare, dar nu avem tipuri de exceptii definite</t>
-  </si>
-  <si>
-    <t xml:space="preserve">A06</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Se foloseste sablould MWC (model view controller)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">A07</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Product,Inventory</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Unele denumiri nu reflecta clar rolul atributelor sau metodelor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Review Form. Coding Defects</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Coding Document</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Popescu Ionel</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Product</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sunt definite metode care nu sunt folosite (lookupAssociatedPart, removeAssociatedPart)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C09</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AddProductController, 150</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Se foloseste obiectul in loc de id pentru functia de stergere</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Inventory Repository</t>
-  </si>
-  <si>
-    <t xml:space="preserve">sunt folosite variabile redundante(br, line, product)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tool-based Code Analysis</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tool used:</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SonarQube</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Iliuță Filip</t>
-  </si>
-  <si>
-    <t xml:space="preserve">17.03.2025</t>
-  </si>
-  <si>
-    <t xml:space="preserve">File, Line</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Issue</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Before</t>
-  </si>
-  <si>
-    <t xml:space="preserve">After/Argument</t>
-  </si>
-  <si>
-    <t xml:space="preserve">InventoryRepository.java, 26</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Resources should be closed java: S2095</t>
+    <t>Georgescu Anca</t>
+  </si>
+  <si>
+    <t>A05</t>
+  </si>
+  <si>
+    <t>In controller exista mesaje de eroare, dar nu avem tipuri de exceptii definite</t>
+  </si>
+  <si>
+    <t>A06</t>
+  </si>
+  <si>
+    <t>Se foloseste sablould MWC (model view controller)</t>
+  </si>
+  <si>
+    <t>A07</t>
+  </si>
+  <si>
+    <t>Product,Inventory</t>
+  </si>
+  <si>
+    <t>Unele denumiri nu reflecta clar rolul atributelor sau metodelor</t>
+  </si>
+  <si>
+    <t>Review Form. Coding Defects</t>
+  </si>
+  <si>
+    <t>Coding Document</t>
+  </si>
+  <si>
+    <t>Popescu Ionel</t>
+  </si>
+  <si>
+    <t>C01</t>
+  </si>
+  <si>
+    <t>Product</t>
+  </si>
+  <si>
+    <t>Sunt definite metode care nu sunt folosite (lookupAssociatedPart, removeAssociatedPart)</t>
+  </si>
+  <si>
+    <t>C09</t>
+  </si>
+  <si>
+    <t>AddProductController, 150</t>
+  </si>
+  <si>
+    <t>Se foloseste obiectul in loc de id pentru functia de stergere</t>
+  </si>
+  <si>
+    <t>Inventory Repository</t>
+  </si>
+  <si>
+    <t>sunt folosite variabile redundante(br, line, product)</t>
+  </si>
+  <si>
+    <t>Tool-based Code Analysis</t>
+  </si>
+  <si>
+    <t>Tool used:</t>
+  </si>
+  <si>
+    <t>SonarQube</t>
+  </si>
+  <si>
+    <t>Iliuță Filip</t>
+  </si>
+  <si>
+    <t>17.03.2025</t>
+  </si>
+  <si>
+    <t>File, Line</t>
+  </si>
+  <si>
+    <t>Issue</t>
+  </si>
+  <si>
+    <t>Before</t>
+  </si>
+  <si>
+    <t>After/Argument</t>
+  </si>
+  <si>
+    <t>InventoryRepository.java, 26</t>
+  </si>
+  <si>
+    <t>Resources should be closed java: S2095</t>
   </si>
   <si>
     <r>
@@ -232,7 +248,7 @@
         <family val="3"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">readParts</t>
+      <t>readParts</t>
     </r>
     <r>
       <rPr>
@@ -284,40 +300,40 @@
         <family val="3"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">File(</t>
-    </r>
-    <r>
-      <rPr>
-        <i val="true"/>
+      <t>File(</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
         <sz val="11.5"/>
         <color rgb="FFC77DBB"/>
         <rFont val="JetBrains Mono"/>
         <family val="3"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">filename</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11.5"/>
-        <color rgb="FFBCBEC4"/>
-        <rFont val="JetBrains Mono"/>
-        <family val="3"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">);
+      <t>filename</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11.5"/>
+        <color rgb="FFBCBEC4"/>
+        <rFont val="JetBrains Mono"/>
+        <family val="3"/>
+        <charset val="1"/>
+      </rPr>
+      <t>);
 	ObservableList&lt;Part&gt; listP = FXCollections.</t>
     </r>
     <r>
       <rPr>
-        <i val="true"/>
-        <sz val="11.5"/>
-        <color rgb="FFBCBEC4"/>
-        <rFont val="JetBrains Mono"/>
-        <family val="3"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">observableArrayList</t>
+        <i/>
+        <sz val="11.5"/>
+        <color rgb="FFBCBEC4"/>
+        <rFont val="JetBrains Mono"/>
+        <family val="3"/>
+        <charset val="1"/>
+      </rPr>
+      <t>observableArrayList</t>
     </r>
     <r>
       <rPr>
@@ -369,7 +385,7 @@
         <family val="3"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">BufferedReader(</t>
+      <t>BufferedReader(</t>
     </r>
     <r>
       <rPr>
@@ -447,17 +463,17 @@
         <family val="3"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">inventory</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11.5"/>
-        <color rgb="FFBCBEC4"/>
-        <rFont val="JetBrains Mono"/>
-        <family val="3"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">.setAllParts(listP);
+      <t>inventory</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11.5"/>
+        <color rgb="FFBCBEC4"/>
+        <rFont val="JetBrains Mono"/>
+        <family val="3"/>
+        <charset val="1"/>
+      </rPr>
+      <t>.setAllParts(listP);
 }</t>
     </r>
   </si>
@@ -480,7 +496,7 @@
         <family val="3"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">readParts</t>
+      <t>readParts</t>
     </r>
     <r>
       <rPr>
@@ -532,40 +548,40 @@
         <family val="3"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">File(</t>
-    </r>
-    <r>
-      <rPr>
-        <i val="true"/>
+      <t>File(</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
         <sz val="11.5"/>
         <color rgb="FFC77DBB"/>
         <rFont val="JetBrains Mono"/>
         <family val="3"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">filename</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11.5"/>
-        <color rgb="FFBCBEC4"/>
-        <rFont val="JetBrains Mono"/>
-        <family val="3"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">);
+      <t>filename</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11.5"/>
+        <color rgb="FFBCBEC4"/>
+        <rFont val="JetBrains Mono"/>
+        <family val="3"/>
+        <charset val="1"/>
+      </rPr>
+      <t>);
 	ObservableList&lt;Part&gt; listP = FXCollections.</t>
     </r>
     <r>
       <rPr>
-        <i val="true"/>
-        <sz val="11.5"/>
-        <color rgb="FFBCBEC4"/>
-        <rFont val="JetBrains Mono"/>
-        <family val="3"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">observableArrayList</t>
+        <i/>
+        <sz val="11.5"/>
+        <color rgb="FFBCBEC4"/>
+        <rFont val="JetBrains Mono"/>
+        <family val="3"/>
+        <charset val="1"/>
+      </rPr>
+      <t>observableArrayList</t>
     </r>
     <r>
       <rPr>
@@ -586,7 +602,7 @@
         <family val="3"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">try</t>
+      <t>try</t>
     </r>
     <r>
       <rPr>
@@ -616,7 +632,7 @@
         <family val="3"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">BufferedReader(</t>
+      <t>BufferedReader(</t>
     </r>
     <r>
       <rPr>
@@ -694,22 +710,22 @@
         <family val="3"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">inventory</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11.5"/>
-        <color rgb="FFBCBEC4"/>
-        <rFont val="JetBrains Mono"/>
-        <family val="3"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">.setAllParts(listP);
+      <t>inventory</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11.5"/>
+        <color rgb="FFBCBEC4"/>
+        <rFont val="JetBrains Mono"/>
+        <family val="3"/>
+        <charset val="1"/>
+      </rPr>
+      <t>.setAllParts(listP);
 }</t>
     </r>
   </si>
   <si>
-    <t xml:space="preserve">InventoryRepository.java, 77</t>
+    <t>InventoryRepository.java, 77</t>
   </si>
   <si>
     <r>
@@ -730,7 +746,7 @@
         <family val="3"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">readProducts</t>
+      <t>readProducts</t>
     </r>
     <r>
       <rPr>
@@ -782,40 +798,40 @@
         <family val="3"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">File(</t>
-    </r>
-    <r>
-      <rPr>
-        <i val="true"/>
+      <t>File(</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
         <sz val="11.5"/>
         <color rgb="FFC77DBB"/>
         <rFont val="JetBrains Mono"/>
         <family val="3"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">filename</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11.5"/>
-        <color rgb="FFBCBEC4"/>
-        <rFont val="JetBrains Mono"/>
-        <family val="3"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">);
+      <t>filename</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11.5"/>
+        <color rgb="FFBCBEC4"/>
+        <rFont val="JetBrains Mono"/>
+        <family val="3"/>
+        <charset val="1"/>
+      </rPr>
+      <t>);
 	ObservableList&lt;Product&gt; listP = FXCollections.</t>
     </r>
     <r>
       <rPr>
-        <i val="true"/>
-        <sz val="11.5"/>
-        <color rgb="FFBCBEC4"/>
-        <rFont val="JetBrains Mono"/>
-        <family val="3"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">observableArrayList</t>
+        <i/>
+        <sz val="11.5"/>
+        <color rgb="FFBCBEC4"/>
+        <rFont val="JetBrains Mono"/>
+        <family val="3"/>
+        <charset val="1"/>
+      </rPr>
+      <t>observableArrayList</t>
     </r>
     <r>
       <rPr>
@@ -867,7 +883,7 @@
         <family val="3"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">BufferedReader(</t>
+      <t>BufferedReader(</t>
     </r>
     <r>
       <rPr>
@@ -945,17 +961,17 @@
         <family val="3"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">inventory</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11.5"/>
-        <color rgb="FFBCBEC4"/>
-        <rFont val="JetBrains Mono"/>
-        <family val="3"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">.setProducts(listP);
+      <t>inventory</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11.5"/>
+        <color rgb="FFBCBEC4"/>
+        <rFont val="JetBrains Mono"/>
+        <family val="3"/>
+        <charset val="1"/>
+      </rPr>
+      <t>.setProducts(listP);
 }</t>
     </r>
   </si>
@@ -978,7 +994,7 @@
         <family val="3"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">readProducts</t>
+      <t>readProducts</t>
     </r>
     <r>
       <rPr>
@@ -1030,40 +1046,40 @@
         <family val="3"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">File(</t>
-    </r>
-    <r>
-      <rPr>
-        <i val="true"/>
+      <t>File(</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
         <sz val="11.5"/>
         <color rgb="FFC77DBB"/>
         <rFont val="JetBrains Mono"/>
         <family val="3"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">filename</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11.5"/>
-        <color rgb="FFBCBEC4"/>
-        <rFont val="JetBrains Mono"/>
-        <family val="3"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">);
+      <t>filename</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11.5"/>
+        <color rgb="FFBCBEC4"/>
+        <rFont val="JetBrains Mono"/>
+        <family val="3"/>
+        <charset val="1"/>
+      </rPr>
+      <t>);
 	ObservableList&lt;Product&gt; listP = FXCollections.</t>
     </r>
     <r>
       <rPr>
-        <i val="true"/>
-        <sz val="11.5"/>
-        <color rgb="FFBCBEC4"/>
-        <rFont val="JetBrains Mono"/>
-        <family val="3"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">observableArrayList</t>
+        <i/>
+        <sz val="11.5"/>
+        <color rgb="FFBCBEC4"/>
+        <rFont val="JetBrains Mono"/>
+        <family val="3"/>
+        <charset val="1"/>
+      </rPr>
+      <t>observableArrayList</t>
     </r>
     <r>
       <rPr>
@@ -1114,7 +1130,7 @@
         <family val="3"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">BufferedReader(</t>
+      <t>BufferedReader(</t>
     </r>
     <r>
       <rPr>
@@ -1192,22 +1208,22 @@
         <family val="3"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">inventory</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11.5"/>
-        <color rgb="FFBCBEC4"/>
-        <rFont val="JetBrains Mono"/>
-        <family val="3"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">.setProducts(listP);
+      <t>inventory</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11.5"/>
+        <color rgb="FFBCBEC4"/>
+        <rFont val="JetBrains Mono"/>
+        <family val="3"/>
+        <charset val="1"/>
+      </rPr>
+      <t>.setProducts(listP);
 }</t>
     </r>
   </si>
   <si>
-    <t xml:space="preserve">InventoryRepository.java, 131</t>
+    <t>InventoryRepository.java, 131</t>
   </si>
   <si>
     <r>
@@ -1228,7 +1244,7 @@
         <family val="3"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">writeAll</t>
+      <t>writeAll</t>
     </r>
     <r>
       <rPr>
@@ -1280,28 +1296,28 @@
         <family val="3"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">File(</t>
-    </r>
-    <r>
-      <rPr>
-        <i val="true"/>
+      <t>File(</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
         <sz val="11.5"/>
         <color rgb="FFC77DBB"/>
         <rFont val="JetBrains Mono"/>
         <family val="3"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">filename</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11.5"/>
-        <color rgb="FFBCBEC4"/>
-        <rFont val="JetBrains Mono"/>
-        <family val="3"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">);
+      <t>filename</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11.5"/>
+        <color rgb="FFBCBEC4"/>
+        <rFont val="JetBrains Mono"/>
+        <family val="3"/>
+        <charset val="1"/>
+      </rPr>
+      <t>);
 	ObservableList&lt;Part&gt; parts=</t>
     </r>
     <r>
@@ -1312,17 +1328,17 @@
         <family val="3"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">inventory</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11.5"/>
-        <color rgb="FFBCBEC4"/>
-        <rFont val="JetBrains Mono"/>
-        <family val="3"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">.getAllParts();
+      <t>inventory</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11.5"/>
+        <color rgb="FFBCBEC4"/>
+        <rFont val="JetBrains Mono"/>
+        <family val="3"/>
+        <charset val="1"/>
+      </rPr>
+      <t>.getAllParts();
 	ObservableList&lt;Product&gt; products=</t>
     </r>
     <r>
@@ -1333,7 +1349,7 @@
         <family val="3"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">inventory</t>
+      <t>inventory</t>
     </r>
     <r>
       <rPr>
@@ -1385,7 +1401,7 @@
         <family val="3"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">BufferedWriter(</t>
+      <t>BufferedWriter(</t>
     </r>
     <r>
       <rPr>
@@ -1428,7 +1444,7 @@
         <family val="3"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">(IOException e) {
+      <t>(IOException e) {
 		e.printStackTrace();
 	}
 }</t>
@@ -1453,7 +1469,7 @@
         <family val="3"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">writeAll</t>
+      <t>writeAll</t>
     </r>
     <r>
       <rPr>
@@ -1505,28 +1521,28 @@
         <family val="3"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">File(</t>
-    </r>
-    <r>
-      <rPr>
-        <i val="true"/>
+      <t>File(</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
         <sz val="11.5"/>
         <color rgb="FFC77DBB"/>
         <rFont val="JetBrains Mono"/>
         <family val="3"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">filename</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11.5"/>
-        <color rgb="FFBCBEC4"/>
-        <rFont val="JetBrains Mono"/>
-        <family val="3"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">);
+      <t>filename</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11.5"/>
+        <color rgb="FFBCBEC4"/>
+        <rFont val="JetBrains Mono"/>
+        <family val="3"/>
+        <charset val="1"/>
+      </rPr>
+      <t>);
 	ObservableList&lt;Part&gt; parts=</t>
     </r>
     <r>
@@ -1537,17 +1553,17 @@
         <family val="3"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">inventory</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11.5"/>
-        <color rgb="FFBCBEC4"/>
-        <rFont val="JetBrains Mono"/>
-        <family val="3"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">.getAllParts();
+      <t>inventory</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11.5"/>
+        <color rgb="FFBCBEC4"/>
+        <rFont val="JetBrains Mono"/>
+        <family val="3"/>
+        <charset val="1"/>
+      </rPr>
+      <t>.getAllParts();
 	ObservableList&lt;Product&gt; products=</t>
     </r>
     <r>
@@ -1558,7 +1574,7 @@
         <family val="3"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">inventory</t>
+      <t>inventory</t>
     </r>
     <r>
       <rPr>
@@ -1609,7 +1625,7 @@
         <family val="3"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">BufferedWriter(</t>
+      <t>BufferedWriter(</t>
     </r>
     <r>
       <rPr>
@@ -1652,17 +1668,17 @@
         <family val="3"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">(IOException e) {
+      <t>(IOException e) {
 		e.printStackTrace();
 	}
 }</t>
     </r>
   </si>
   <si>
-    <t xml:space="preserve">Product.java, 60</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Variables should not be self-assigned, java: S1656</t>
+    <t>Product.java, 60</t>
+  </si>
+  <si>
+    <t>Variables should not be self-assigned, java: S1656</t>
   </si>
   <si>
     <r>
@@ -1683,17 +1699,17 @@
         <family val="3"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">setAssociatedParts</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11.5"/>
-        <color rgb="FFBCBEC4"/>
-        <rFont val="JetBrains Mono"/>
-        <family val="3"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">(ObservableList&lt;Part&gt; associatedParts) {
+      <t>setAssociatedParts</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11.5"/>
+        <color rgb="FFBCBEC4"/>
+        <rFont val="JetBrains Mono"/>
+        <family val="3"/>
+        <charset val="1"/>
+      </rPr>
+      <t>(ObservableList&lt;Part&gt; associatedParts) {
     associatedParts = associatedParts;
 }</t>
     </r>
@@ -1717,7 +1733,7 @@
         <family val="3"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">setAssociatedParts</t>
+      <t>setAssociatedParts</t>
     </r>
     <r>
       <rPr>
@@ -1738,17 +1754,17 @@
         <family val="3"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">this</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11.5"/>
-        <color rgb="FFBCBEC4"/>
-        <rFont val="JetBrains Mono"/>
-        <family val="3"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">.</t>
+      <t>this</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11.5"/>
+        <color rgb="FFBCBEC4"/>
+        <rFont val="JetBrains Mono"/>
+        <family val="3"/>
+        <charset val="1"/>
+      </rPr>
+      <t>.</t>
     </r>
     <r>
       <rPr>
@@ -1768,15 +1784,15 @@
         <family val="3"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">= associatedParts;
+      <t>= associatedParts;
 }</t>
     </r>
   </si>
   <si>
-    <t xml:space="preserve">Part.java, 18</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Constructors of an "abstract" class should not be declared "public", java: S5993</t>
+    <t>Part.java, 18</t>
+  </si>
+  <si>
+    <t>Constructors of an "abstract" class should not be declared "public", java: S5993</t>
   </si>
   <si>
     <r>
@@ -1797,17 +1813,17 @@
         <family val="3"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">Part</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11.5"/>
-        <color rgb="FFBCBEC4"/>
-        <rFont val="JetBrains Mono"/>
-        <family val="3"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">(</t>
+      <t>Part</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11.5"/>
+        <color rgb="FFBCBEC4"/>
+        <rFont val="JetBrains Mono"/>
+        <family val="3"/>
+        <charset val="1"/>
+      </rPr>
+      <t>(</t>
     </r>
     <r>
       <rPr>
@@ -1918,17 +1934,17 @@
         <family val="3"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">this</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11.5"/>
-        <color rgb="FFBCBEC4"/>
-        <rFont val="JetBrains Mono"/>
-        <family val="3"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">.</t>
+      <t>this</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11.5"/>
+        <color rgb="FFBCBEC4"/>
+        <rFont val="JetBrains Mono"/>
+        <family val="3"/>
+        <charset val="1"/>
+      </rPr>
+      <t>.</t>
     </r>
     <r>
       <rPr>
@@ -1959,17 +1975,17 @@
         <family val="3"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">this</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11.5"/>
-        <color rgb="FFBCBEC4"/>
-        <rFont val="JetBrains Mono"/>
-        <family val="3"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">.</t>
+      <t>this</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11.5"/>
+        <color rgb="FFBCBEC4"/>
+        <rFont val="JetBrains Mono"/>
+        <family val="3"/>
+        <charset val="1"/>
+      </rPr>
+      <t>.</t>
     </r>
     <r>
       <rPr>
@@ -2000,17 +2016,17 @@
         <family val="3"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">this</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11.5"/>
-        <color rgb="FFBCBEC4"/>
-        <rFont val="JetBrains Mono"/>
-        <family val="3"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">.</t>
+      <t>this</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11.5"/>
+        <color rgb="FFBCBEC4"/>
+        <rFont val="JetBrains Mono"/>
+        <family val="3"/>
+        <charset val="1"/>
+      </rPr>
+      <t>.</t>
     </r>
     <r>
       <rPr>
@@ -2041,17 +2057,17 @@
         <family val="3"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">this</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11.5"/>
-        <color rgb="FFBCBEC4"/>
-        <rFont val="JetBrains Mono"/>
-        <family val="3"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">.</t>
+      <t>this</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11.5"/>
+        <color rgb="FFBCBEC4"/>
+        <rFont val="JetBrains Mono"/>
+        <family val="3"/>
+        <charset val="1"/>
+      </rPr>
+      <t>.</t>
     </r>
     <r>
       <rPr>
@@ -2082,17 +2098,17 @@
         <family val="3"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">this</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11.5"/>
-        <color rgb="FFBCBEC4"/>
-        <rFont val="JetBrains Mono"/>
-        <family val="3"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">.</t>
+      <t>this</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11.5"/>
+        <color rgb="FFBCBEC4"/>
+        <rFont val="JetBrains Mono"/>
+        <family val="3"/>
+        <charset val="1"/>
+      </rPr>
+      <t>.</t>
     </r>
     <r>
       <rPr>
@@ -2123,17 +2139,17 @@
         <family val="3"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">this</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11.5"/>
-        <color rgb="FFBCBEC4"/>
-        <rFont val="JetBrains Mono"/>
-        <family val="3"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">.</t>
+      <t>this</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11.5"/>
+        <color rgb="FFBCBEC4"/>
+        <rFont val="JetBrains Mono"/>
+        <family val="3"/>
+        <charset val="1"/>
+      </rPr>
+      <t>.</t>
     </r>
     <r>
       <rPr>
@@ -2153,7 +2169,7 @@
         <family val="3"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">= max;
+      <t>= max;
 }</t>
     </r>
   </si>
@@ -2176,17 +2192,17 @@
         <family val="3"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">Part</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11.5"/>
-        <color rgb="FFBCBEC4"/>
-        <rFont val="JetBrains Mono"/>
-        <family val="3"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">(</t>
+      <t>Part</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11.5"/>
+        <color rgb="FFBCBEC4"/>
+        <rFont val="JetBrains Mono"/>
+        <family val="3"/>
+        <charset val="1"/>
+      </rPr>
+      <t>(</t>
     </r>
     <r>
       <rPr>
@@ -2297,17 +2313,17 @@
         <family val="3"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">this</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11.5"/>
-        <color rgb="FFBCBEC4"/>
-        <rFont val="JetBrains Mono"/>
-        <family val="3"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">.</t>
+      <t>this</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11.5"/>
+        <color rgb="FFBCBEC4"/>
+        <rFont val="JetBrains Mono"/>
+        <family val="3"/>
+        <charset val="1"/>
+      </rPr>
+      <t>.</t>
     </r>
     <r>
       <rPr>
@@ -2338,17 +2354,17 @@
         <family val="3"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">this</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11.5"/>
-        <color rgb="FFBCBEC4"/>
-        <rFont val="JetBrains Mono"/>
-        <family val="3"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">.</t>
+      <t>this</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11.5"/>
+        <color rgb="FFBCBEC4"/>
+        <rFont val="JetBrains Mono"/>
+        <family val="3"/>
+        <charset val="1"/>
+      </rPr>
+      <t>.</t>
     </r>
     <r>
       <rPr>
@@ -2379,17 +2395,17 @@
         <family val="3"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">this</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11.5"/>
-        <color rgb="FFBCBEC4"/>
-        <rFont val="JetBrains Mono"/>
-        <family val="3"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">.</t>
+      <t>this</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11.5"/>
+        <color rgb="FFBCBEC4"/>
+        <rFont val="JetBrains Mono"/>
+        <family val="3"/>
+        <charset val="1"/>
+      </rPr>
+      <t>.</t>
     </r>
     <r>
       <rPr>
@@ -2420,17 +2436,17 @@
         <family val="3"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">this</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11.5"/>
-        <color rgb="FFBCBEC4"/>
-        <rFont val="JetBrains Mono"/>
-        <family val="3"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">.</t>
+      <t>this</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11.5"/>
+        <color rgb="FFBCBEC4"/>
+        <rFont val="JetBrains Mono"/>
+        <family val="3"/>
+        <charset val="1"/>
+      </rPr>
+      <t>.</t>
     </r>
     <r>
       <rPr>
@@ -2461,17 +2477,17 @@
         <family val="3"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">this</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11.5"/>
-        <color rgb="FFBCBEC4"/>
-        <rFont val="JetBrains Mono"/>
-        <family val="3"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">.</t>
+      <t>this</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11.5"/>
+        <color rgb="FFBCBEC4"/>
+        <rFont val="JetBrains Mono"/>
+        <family val="3"/>
+        <charset val="1"/>
+      </rPr>
+      <t>.</t>
     </r>
     <r>
       <rPr>
@@ -2502,17 +2518,17 @@
         <family val="3"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">this</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11.5"/>
-        <color rgb="FFBCBEC4"/>
-        <rFont val="JetBrains Mono"/>
-        <family val="3"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">.</t>
+      <t>this</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11.5"/>
+        <color rgb="FFBCBEC4"/>
+        <rFont val="JetBrains Mono"/>
+        <family val="3"/>
+        <charset val="1"/>
+      </rPr>
+      <t>.</t>
     </r>
     <r>
       <rPr>
@@ -2532,15 +2548,15 @@
         <family val="3"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">= max;
+      <t>= max;
 }</t>
     </r>
   </si>
   <si>
-    <t xml:space="preserve">AddProductController.java, 31</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Constructors should not be used to instantiate "String", "BigInteger", "BigDecimal" and primitive-wrapper, java: S2129</t>
+    <t>AddProductController.java, 31</t>
+  </si>
+  <si>
+    <t>Constructors should not be used to instantiate "String", "BigInteger", "BigDecimal" and primitive-wrapper, java: S2129</t>
   </si>
   <si>
     <r>
@@ -2595,7 +2611,7 @@
         <rFont val="JetBrains Mono"/>
         <family val="3"/>
       </rPr>
-      <t xml:space="preserve">String();</t>
+      <t>String();</t>
     </r>
   </si>
   <si>
@@ -2642,7 +2658,7 @@
         <rFont val="JetBrains Mono"/>
         <family val="3"/>
       </rPr>
-      <t xml:space="preserve">""</t>
+      <t>""</t>
     </r>
     <r>
       <rPr>
@@ -2656,10 +2672,10 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">AddProductController.java, 32</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Unused "private" fields should be removed, java: S1068</t>
+    <t>AddProductController.java, 32</t>
+  </si>
+  <si>
+    <t>Unused "private" fields should be removed, java: S1068</t>
   </si>
   <si>
     <r>
@@ -2678,54 +2694,36 @@
         <rFont val="JetBrains Mono"/>
         <family val="3"/>
       </rPr>
-      <t xml:space="preserve">productId</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11.5"/>
-        <color rgb="FFBCBEC4"/>
-        <rFont val="JetBrains Mono"/>
-        <family val="3"/>
-      </rPr>
-      <t xml:space="preserve">;</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">[unused  private field removed]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Effort to perform tool-based code analysis (hours): 0.5</t>
+      <t>productId</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11.5"/>
+        <color rgb="FFBCBEC4"/>
+        <rFont val="JetBrains Mono"/>
+        <family val="3"/>
+      </rPr>
+      <t>;</t>
+    </r>
+  </si>
+  <si>
+    <t>[unused  private field removed]</t>
+  </si>
+  <si>
+    <t>Effort to perform tool-based code analysis (hours): 0.5</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="General"/>
-  </numFmts>
-  <fonts count="21">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="18">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="238"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
     </font>
     <font>
       <sz val="11"/>
@@ -2735,7 +2733,7 @@
       <charset val="1"/>
     </font>
     <font>
-      <b val="true"/>
+      <b/>
       <sz val="12"/>
       <color rgb="FF000080"/>
       <name val="Calibri"/>
@@ -2743,7 +2741,7 @@
       <charset val="1"/>
     </font>
     <font>
-      <i val="true"/>
+      <i/>
       <sz val="9"/>
       <color rgb="FFC00000"/>
       <name val="Calibri"/>
@@ -2751,7 +2749,7 @@
       <charset val="1"/>
     </font>
     <font>
-      <b val="true"/>
+      <b/>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
@@ -2759,8 +2757,8 @@
       <charset val="1"/>
     </font>
     <font>
-      <b val="true"/>
-      <i val="true"/>
+      <b/>
+      <i/>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
@@ -2768,7 +2766,7 @@
       <charset val="1"/>
     </font>
     <font>
-      <i val="true"/>
+      <i/>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
@@ -2804,7 +2802,7 @@
       <charset val="1"/>
     </font>
     <font>
-      <i val="true"/>
+      <i/>
       <sz val="11.5"/>
       <color rgb="FFC77DBB"/>
       <name val="JetBrains Mono"/>
@@ -2812,7 +2810,7 @@
       <charset val="1"/>
     </font>
     <font>
-      <i val="true"/>
+      <i/>
       <sz val="11.5"/>
       <color rgb="FFBCBEC4"/>
       <name val="JetBrains Mono"/>
@@ -2878,209 +2876,141 @@
     </fill>
   </fills>
   <borders count="5">
-    <border diagonalUp="false" diagonalDown="false">
+    <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
       <diagonal/>
     </border>
-    <border diagonalUp="false" diagonalDown="false">
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
-    <border diagonalUp="false" diagonalDown="false">
-      <left style="thin"/>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
       <right/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
-    <border diagonalUp="false" diagonalDown="false">
+    <border>
       <left/>
       <right/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
-    <border diagonalUp="false" diagonalDown="false">
-      <left style="thin"/>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
       <right/>
       <top/>
       <bottom/>
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="20">
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+  <cellStyleXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="33">
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="6">
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Comma" xfId="15" builtinId="3"/>
-    <cellStyle name="Comma [0]" xfId="16" builtinId="6"/>
-    <cellStyle name="Currency" xfId="17" builtinId="4"/>
-    <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
-    <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
+  <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="FF000000"/>
@@ -3139,1368 +3069,1699 @@
       <rgbColor rgb="FF993366"/>
       <rgbColor rgb="FF333399"/>
       <rgbColor rgb="FF333333"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
     </indexedColors>
   </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+  <a:themeElements>
+    <a:clrScheme name="Office">
+      <a:dk1>
+        <a:sysClr val="windowText" lastClr="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="0E2841"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="E8E8E8"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="156082"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="E97132"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="196B24"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="0F9ED5"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="A02B93"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="4EA72E"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="467886"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="96607D"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Aptos Display" panose="02110004020202020204"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="游ゴシック Light"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="等线 Light"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="游ゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="等线"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme name="Office">
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="110000"/>
+                <a:satMod val="105000"/>
+                <a:tint val="67000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="105000"/>
+                <a:satMod val="103000"/>
+                <a:tint val="73000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="105000"/>
+                <a:satMod val="109000"/>
+                <a:tint val="81000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:satMod val="103000"/>
+                <a:lumMod val="102000"/>
+                <a:tint val="94000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="phClr">
+                <a:satMod val="110000"/>
+                <a:lumMod val="100000"/>
+                <a:shade val="100000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="99000"/>
+                <a:satMod val="120000"/>
+                <a:shade val="78000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="63000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr">
+            <a:tint val="95000"/>
+            <a:satMod val="170000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="93000"/>
+                <a:satMod val="150000"/>
+                <a:shade val="98000"/>
+                <a:lumMod val="102000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="phClr">
+                <a:tint val="98000"/>
+                <a:satMod val="130000"/>
+                <a:shade val="90000"/>
+                <a:lumMod val="103000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="63000"/>
+                <a:satMod val="120000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+  <a:objectDefaults>
+    <a:lnDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </a:style>
+    </a:lnDef>
+  </a:objectDefaults>
+  <a:extraClrSchemeLst/>
+  <a:extLst>
+    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
+    </a:ext>
+  </a:extLst>
+</a:theme>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr>
     <tabColor rgb="FFCCC1DA"/>
-    <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:J27"/>
-  <sheetFormatPr defaultColWidth="8.90234375" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:AMJ27"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="8.89"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="12.22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="1" width="16.22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="41.44"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="8" min="6" style="1" width="8.89"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="20.98"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="14.43"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1024" min="11" style="1" width="8.89"/>
+    <col min="1" max="1" width="8.88671875" style="11"/>
+    <col min="2" max="2" width="12.21875" style="11" customWidth="1"/>
+    <col min="3" max="4" width="16.21875" style="11" customWidth="1"/>
+    <col min="5" max="5" width="41.44140625" style="11" customWidth="1"/>
+    <col min="6" max="8" width="8.88671875" style="11"/>
+    <col min="9" max="9" width="21" style="11" customWidth="1"/>
+    <col min="10" max="10" width="14.44140625" style="11" customWidth="1"/>
+    <col min="11" max="1024" width="8.88671875" style="11"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2"/>
-      <c r="B1" s="3" t="s">
+    <row r="1" spans="1:10" ht="15.6">
+      <c r="A1" s="12"/>
+      <c r="B1" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="H1" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="I1" s="4"/>
-      <c r="J1" s="4"/>
-    </row>
-    <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B2" s="5" t="s">
+      <c r="I1" s="10"/>
+      <c r="J1" s="10"/>
+    </row>
+    <row r="2" spans="1:10">
+      <c r="B2" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="5"/>
-      <c r="D2" s="5"/>
-      <c r="E2" s="5"/>
-      <c r="H2" s="6"/>
-      <c r="I2" s="6" t="s">
+      <c r="C2" s="9"/>
+      <c r="D2" s="9"/>
+      <c r="E2" s="9"/>
+      <c r="H2" s="14"/>
+      <c r="I2" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="J2" s="6" t="s">
+      <c r="J2" s="14" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H3" s="6" t="s">
+    <row r="3" spans="1:10">
+      <c r="H3" s="14" t="s">
         <v>5</v>
       </c>
-      <c r="I3" s="6" t="s">
+      <c r="I3" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="J3" s="6" t="n">
+      <c r="J3" s="14">
         <v>233</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C4" s="7" t="s">
+    <row r="4" spans="1:10">
+      <c r="C4" s="15" t="s">
         <v>7</v>
       </c>
       <c r="D4" s="8" t="s">
         <v>8</v>
       </c>
       <c r="E4" s="8"/>
-      <c r="H4" s="6" t="s">
+      <c r="H4" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="I4" s="6" t="s">
+      <c r="I4" s="14" t="s">
         <v>10</v>
       </c>
-      <c r="J4" s="6" t="n">
+      <c r="J4" s="14">
         <v>233</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C5" s="7" t="s">
+    <row r="5" spans="1:10">
+      <c r="C5" s="15" t="s">
         <v>11</v>
       </c>
-      <c r="D5" s="9" t="s">
+      <c r="D5" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="9"/>
-      <c r="H5" s="6" t="s">
+      <c r="E5" s="7"/>
+      <c r="H5" s="14" t="s">
         <v>13</v>
       </c>
-      <c r="I5" s="6" t="s">
+      <c r="I5" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="J5" s="6" t="n">
+      <c r="J5" s="14">
         <v>233</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B6" s="10"/>
-      <c r="C6" s="11" t="s">
+    <row r="6" spans="1:10">
+      <c r="B6" s="16"/>
+      <c r="C6" s="17" t="s">
         <v>15</v>
       </c>
-      <c r="D6" s="12"/>
-      <c r="E6" s="12"/>
-    </row>
-    <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C7" s="11" t="s">
+      <c r="D6" s="6"/>
+      <c r="E6" s="6"/>
+    </row>
+    <row r="7" spans="1:10">
+      <c r="C7" s="17" t="s">
         <v>16</v>
       </c>
-      <c r="D7" s="12" t="s">
+      <c r="D7" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="E7" s="12"/>
-    </row>
-    <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B9" s="13" t="s">
+      <c r="E7" s="6"/>
+    </row>
+    <row r="9" spans="1:10">
+      <c r="B9" s="18" t="s">
         <v>18</v>
       </c>
-      <c r="C9" s="13" t="s">
+      <c r="C9" s="18" t="s">
         <v>19</v>
       </c>
-      <c r="D9" s="13" t="s">
+      <c r="D9" s="18" t="s">
         <v>20</v>
       </c>
-      <c r="E9" s="14" t="s">
+      <c r="E9" s="19" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="72" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B10" s="6" t="n">
+    <row r="10" spans="1:10" ht="72">
+      <c r="B10" s="14">
         <v>1</v>
       </c>
-      <c r="C10" s="15" t="s">
+      <c r="C10" s="20" t="s">
         <v>22</v>
       </c>
-      <c r="D10" s="15" t="s">
+      <c r="D10" s="20" t="s">
         <v>23</v>
       </c>
-      <c r="E10" s="16" t="s">
+      <c r="E10" s="21" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="28.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B11" s="6" t="n">
-        <f aca="false">B10+1</f>
+    <row r="11" spans="1:10" ht="28.8">
+      <c r="B11" s="14">
+        <f t="shared" ref="B11:B25" si="0">B10+1</f>
         <v>2</v>
       </c>
-      <c r="C11" s="15" t="s">
+      <c r="C11" s="20" t="s">
         <v>25</v>
       </c>
-      <c r="D11" s="15"/>
-      <c r="E11" s="16" t="s">
+      <c r="D11" s="20"/>
+      <c r="E11" s="21" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="28.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B12" s="6" t="n">
-        <f aca="false">B11+1</f>
+    <row r="12" spans="1:10" ht="28.8">
+      <c r="B12" s="14">
+        <f t="shared" si="0"/>
         <v>3</v>
       </c>
-      <c r="C12" s="15" t="s">
+      <c r="C12" s="20" t="s">
         <v>27</v>
       </c>
-      <c r="D12" s="15"/>
-      <c r="E12" s="16" t="s">
+      <c r="D12" s="20"/>
+      <c r="E12" s="21" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B13" s="6" t="n">
-        <f aca="false">B12+1</f>
+    <row r="13" spans="1:10">
+      <c r="B13" s="14">
+        <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="C13" s="15"/>
-      <c r="D13" s="15"/>
-      <c r="E13" s="16"/>
-    </row>
-    <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B14" s="6" t="n">
-        <f aca="false">B13+1</f>
+      <c r="C13" s="20"/>
+      <c r="D13" s="20"/>
+      <c r="E13" s="21"/>
+    </row>
+    <row r="14" spans="1:10">
+      <c r="B14" s="14">
+        <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="C14" s="15"/>
-      <c r="D14" s="15"/>
-      <c r="E14" s="16"/>
-    </row>
-    <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B15" s="6" t="n">
-        <f aca="false">B14+1</f>
+      <c r="C14" s="20"/>
+      <c r="D14" s="20"/>
+      <c r="E14" s="21"/>
+    </row>
+    <row r="15" spans="1:10">
+      <c r="B15" s="14">
+        <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="C15" s="15"/>
-      <c r="D15" s="15"/>
-      <c r="E15" s="16"/>
-    </row>
-    <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B16" s="6" t="n">
-        <f aca="false">B15+1</f>
+      <c r="C15" s="20"/>
+      <c r="D15" s="20"/>
+      <c r="E15" s="21"/>
+    </row>
+    <row r="16" spans="1:10">
+      <c r="B16" s="14">
+        <f t="shared" si="0"/>
         <v>7</v>
       </c>
-      <c r="C16" s="15"/>
-      <c r="D16" s="15"/>
-      <c r="E16" s="16"/>
-    </row>
-    <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B17" s="6" t="n">
-        <f aca="false">B16+1</f>
+      <c r="C16" s="20"/>
+      <c r="D16" s="20"/>
+      <c r="E16" s="21"/>
+    </row>
+    <row r="17" spans="2:5">
+      <c r="B17" s="14">
+        <f t="shared" si="0"/>
         <v>8</v>
       </c>
-      <c r="C17" s="15"/>
-      <c r="D17" s="15"/>
-      <c r="E17" s="16"/>
-    </row>
-    <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B18" s="6" t="n">
-        <f aca="false">B17+1</f>
+      <c r="C17" s="20"/>
+      <c r="D17" s="20"/>
+      <c r="E17" s="21"/>
+    </row>
+    <row r="18" spans="2:5">
+      <c r="B18" s="14">
+        <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="C18" s="6"/>
-      <c r="D18" s="6"/>
-      <c r="E18" s="17"/>
-    </row>
-    <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B19" s="6" t="n">
-        <f aca="false">B18+1</f>
+      <c r="C18" s="14"/>
+      <c r="D18" s="14"/>
+      <c r="E18" s="22"/>
+    </row>
+    <row r="19" spans="2:5">
+      <c r="B19" s="14">
+        <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="C19" s="6"/>
-      <c r="D19" s="6"/>
-      <c r="E19" s="17"/>
-    </row>
-    <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B20" s="6" t="n">
-        <f aca="false">B19+1</f>
+      <c r="C19" s="14"/>
+      <c r="D19" s="14"/>
+      <c r="E19" s="22"/>
+    </row>
+    <row r="20" spans="2:5">
+      <c r="B20" s="14">
+        <f t="shared" si="0"/>
         <v>11</v>
       </c>
-      <c r="C20" s="6"/>
-      <c r="D20" s="6"/>
-      <c r="E20" s="17"/>
-    </row>
-    <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B21" s="6" t="n">
-        <f aca="false">B20+1</f>
+      <c r="C20" s="14"/>
+      <c r="D20" s="14"/>
+      <c r="E20" s="22"/>
+    </row>
+    <row r="21" spans="2:5">
+      <c r="B21" s="14">
+        <f t="shared" si="0"/>
         <v>12</v>
       </c>
-      <c r="C21" s="6"/>
-      <c r="D21" s="6"/>
-      <c r="E21" s="17"/>
-    </row>
-    <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B22" s="6" t="n">
-        <f aca="false">B21+1</f>
+      <c r="C21" s="14"/>
+      <c r="D21" s="14"/>
+      <c r="E21" s="22"/>
+    </row>
+    <row r="22" spans="2:5">
+      <c r="B22" s="14">
+        <f t="shared" si="0"/>
         <v>13</v>
       </c>
-      <c r="C22" s="6"/>
-      <c r="D22" s="6"/>
-      <c r="E22" s="17"/>
-    </row>
-    <row r="23" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B23" s="6" t="n">
-        <f aca="false">B22+1</f>
+      <c r="C22" s="14"/>
+      <c r="D22" s="14"/>
+      <c r="E22" s="22"/>
+    </row>
+    <row r="23" spans="2:5">
+      <c r="B23" s="14">
+        <f t="shared" si="0"/>
         <v>14</v>
       </c>
-      <c r="C23" s="6"/>
-      <c r="D23" s="6"/>
-      <c r="E23" s="17"/>
-    </row>
-    <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B24" s="6" t="n">
-        <f aca="false">B23+1</f>
+      <c r="C23" s="14"/>
+      <c r="D23" s="14"/>
+      <c r="E23" s="22"/>
+    </row>
+    <row r="24" spans="2:5">
+      <c r="B24" s="14">
+        <f t="shared" si="0"/>
         <v>15</v>
       </c>
-      <c r="C24" s="6"/>
-      <c r="D24" s="6"/>
-      <c r="E24" s="17"/>
-    </row>
-    <row r="25" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B25" s="6" t="n">
-        <f aca="false">B24+1</f>
+      <c r="C24" s="14"/>
+      <c r="D24" s="14"/>
+      <c r="E24" s="22"/>
+    </row>
+    <row r="25" spans="2:5">
+      <c r="B25" s="14">
+        <f t="shared" si="0"/>
         <v>16</v>
       </c>
-      <c r="C25" s="6"/>
-      <c r="D25" s="6"/>
-      <c r="E25" s="17"/>
-    </row>
-    <row r="27" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C27" s="18" t="s">
+      <c r="C25" s="14"/>
+      <c r="D25" s="14"/>
+      <c r="E25" s="22"/>
+    </row>
+    <row r="27" spans="2:5">
+      <c r="C27" s="23" t="s">
         <v>29</v>
       </c>
-      <c r="D27" s="19"/>
-      <c r="E27" s="15"/>
+      <c r="D27" s="24"/>
+      <c r="E27" s="20"/>
     </row>
   </sheetData>
   <mergeCells count="6">
+    <mergeCell ref="D7:E7"/>
     <mergeCell ref="H1:J1"/>
     <mergeCell ref="B2:E2"/>
     <mergeCell ref="D4:E4"/>
     <mergeCell ref="D5:E5"/>
     <mergeCell ref="D6:E6"/>
-    <mergeCell ref="D7:E7"/>
   </mergeCells>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <sheetPr>
     <tabColor rgb="FFFCD5B5"/>
-    <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:J28"/>
-  <sheetFormatPr defaultColWidth="8.90234375" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:AMJ28"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="8.89"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="12.22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="1" width="16.22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="41.44"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="8" min="6" style="1" width="8.89"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="22.11"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1024" min="10" style="1" width="8.89"/>
+    <col min="1" max="1" width="8.88671875" style="11"/>
+    <col min="2" max="2" width="12.21875" style="11" customWidth="1"/>
+    <col min="3" max="4" width="16.21875" style="11" customWidth="1"/>
+    <col min="5" max="5" width="41.44140625" style="11" customWidth="1"/>
+    <col min="6" max="8" width="8.88671875" style="11"/>
+    <col min="9" max="9" width="22.109375" style="11" customWidth="1"/>
+    <col min="10" max="1024" width="8.88671875" style="11"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2"/>
-      <c r="B1" s="3" t="s">
+    <row r="1" spans="1:10" ht="15.6">
+      <c r="A1" s="12"/>
+      <c r="B1" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="H1" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="I1" s="4"/>
-      <c r="J1" s="4"/>
-    </row>
-    <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B2" s="5" t="s">
+      <c r="I1" s="10"/>
+      <c r="J1" s="10"/>
+    </row>
+    <row r="2" spans="1:10">
+      <c r="B2" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="C2" s="5"/>
-      <c r="D2" s="5"/>
-      <c r="E2" s="5"/>
-      <c r="H2" s="6"/>
-      <c r="I2" s="6" t="s">
+      <c r="C2" s="9"/>
+      <c r="D2" s="9"/>
+      <c r="E2" s="9"/>
+      <c r="H2" s="14"/>
+      <c r="I2" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="J2" s="6" t="s">
+      <c r="J2" s="14" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H3" s="6" t="s">
+    <row r="3" spans="1:10">
+      <c r="H3" s="14" t="s">
         <v>5</v>
       </c>
-      <c r="I3" s="6" t="s">
+      <c r="I3" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="J3" s="6" t="n">
+      <c r="J3" s="14">
         <v>233</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C4" s="20" t="s">
+    <row r="4" spans="1:10">
+      <c r="C4" s="25" t="s">
         <v>7</v>
       </c>
-      <c r="D4" s="21" t="s">
+      <c r="D4" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="E4" s="21"/>
-      <c r="H4" s="6" t="s">
+      <c r="E4" s="5"/>
+      <c r="H4" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="I4" s="6" t="s">
+      <c r="I4" s="14" t="s">
         <v>10</v>
       </c>
-      <c r="J4" s="6" t="n">
+      <c r="J4" s="14">
         <v>233</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C5" s="20" t="s">
+    <row r="5" spans="1:10">
+      <c r="C5" s="25" t="s">
         <v>32</v>
       </c>
-      <c r="D5" s="22" t="s">
+      <c r="D5" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="E5" s="22"/>
-      <c r="H5" s="6" t="s">
+      <c r="E5" s="4"/>
+      <c r="H5" s="14" t="s">
         <v>13</v>
       </c>
-      <c r="I5" s="6" t="s">
+      <c r="I5" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="J5" s="6" t="n">
+      <c r="J5" s="14">
         <v>233</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B6" s="10"/>
-      <c r="C6" s="11" t="s">
+    <row r="6" spans="1:10">
+      <c r="B6" s="16"/>
+      <c r="C6" s="17" t="s">
         <v>15</v>
       </c>
-      <c r="D6" s="12"/>
-      <c r="E6" s="12"/>
-    </row>
-    <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C7" s="11" t="s">
+      <c r="D6" s="6"/>
+      <c r="E6" s="6"/>
+    </row>
+    <row r="7" spans="1:10">
+      <c r="C7" s="17" t="s">
         <v>16</v>
       </c>
-      <c r="D7" s="12" t="s">
+      <c r="D7" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="E7" s="12"/>
-    </row>
-    <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B9" s="13" t="s">
+      <c r="E7" s="6"/>
+    </row>
+    <row r="9" spans="1:10">
+      <c r="B9" s="18" t="s">
         <v>18</v>
       </c>
-      <c r="C9" s="13" t="s">
+      <c r="C9" s="18" t="s">
         <v>19</v>
       </c>
-      <c r="D9" s="13" t="s">
+      <c r="D9" s="18" t="s">
         <v>20</v>
       </c>
-      <c r="E9" s="13" t="s">
+      <c r="E9" s="18" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="28.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B10" s="6" t="n">
+    <row r="10" spans="1:10" ht="28.8">
+      <c r="B10" s="14">
         <v>1</v>
       </c>
-      <c r="C10" s="15" t="s">
+      <c r="C10" s="20" t="s">
         <v>34</v>
       </c>
-      <c r="D10" s="16"/>
-      <c r="E10" s="16" t="s">
+      <c r="D10" s="21"/>
+      <c r="E10" s="21" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="28.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B11" s="6" t="n">
-        <f aca="false">B10+1</f>
+    <row r="11" spans="1:10" ht="28.8">
+      <c r="B11" s="14">
+        <f t="shared" ref="B11:B26" si="0">B10+1</f>
         <v>2</v>
       </c>
-      <c r="C11" s="15" t="s">
+      <c r="C11" s="20" t="s">
         <v>36</v>
       </c>
-      <c r="D11" s="16"/>
-      <c r="E11" s="16" t="s">
+      <c r="D11" s="21"/>
+      <c r="E11" s="21" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="28.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B12" s="6" t="n">
-        <f aca="false">B11+1</f>
+    <row r="12" spans="1:10" ht="28.8">
+      <c r="B12" s="14">
+        <f t="shared" si="0"/>
         <v>3</v>
       </c>
-      <c r="C12" s="15" t="s">
+      <c r="C12" s="20" t="s">
         <v>38</v>
       </c>
-      <c r="D12" s="15" t="s">
+      <c r="D12" s="20" t="s">
         <v>39</v>
       </c>
-      <c r="E12" s="16" t="s">
+      <c r="E12" s="21" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B13" s="6" t="n">
-        <f aca="false">B12+1</f>
+    <row r="13" spans="1:10">
+      <c r="B13" s="14">
+        <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="C13" s="15"/>
-      <c r="D13" s="15"/>
-      <c r="E13" s="16"/>
-    </row>
-    <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B14" s="6" t="n">
-        <f aca="false">B13+1</f>
+      <c r="C13" s="20"/>
+      <c r="D13" s="20"/>
+      <c r="E13" s="21"/>
+    </row>
+    <row r="14" spans="1:10">
+      <c r="B14" s="14">
+        <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="C14" s="15"/>
-      <c r="D14" s="16"/>
-      <c r="E14" s="16"/>
-    </row>
-    <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B15" s="6" t="n">
-        <f aca="false">B14+1</f>
+      <c r="C14" s="20"/>
+      <c r="D14" s="21"/>
+      <c r="E14" s="21"/>
+    </row>
+    <row r="15" spans="1:10">
+      <c r="B15" s="14">
+        <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="C15" s="15"/>
-      <c r="D15" s="15"/>
-      <c r="E15" s="16"/>
-    </row>
-    <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B16" s="6" t="n">
-        <f aca="false">B15+1</f>
+      <c r="C15" s="20"/>
+      <c r="D15" s="20"/>
+      <c r="E15" s="21"/>
+    </row>
+    <row r="16" spans="1:10">
+      <c r="B16" s="14">
+        <f t="shared" si="0"/>
         <v>7</v>
       </c>
-      <c r="C16" s="15"/>
-      <c r="D16" s="16"/>
-      <c r="E16" s="16"/>
-    </row>
-    <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B17" s="6" t="n">
-        <f aca="false">B16+1</f>
+      <c r="C16" s="20"/>
+      <c r="D16" s="21"/>
+      <c r="E16" s="21"/>
+    </row>
+    <row r="17" spans="2:5">
+      <c r="B17" s="14">
+        <f t="shared" si="0"/>
         <v>8</v>
       </c>
-      <c r="C17" s="15"/>
-      <c r="D17" s="16"/>
-      <c r="E17" s="16"/>
-    </row>
-    <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B18" s="6" t="n">
-        <f aca="false">B17+1</f>
+      <c r="C17" s="20"/>
+      <c r="D17" s="21"/>
+      <c r="E17" s="21"/>
+    </row>
+    <row r="18" spans="2:5">
+      <c r="B18" s="14">
+        <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="C18" s="15"/>
-      <c r="D18" s="15"/>
-      <c r="E18" s="16"/>
-    </row>
-    <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B19" s="6" t="n">
-        <f aca="false">B18+1</f>
+      <c r="C18" s="20"/>
+      <c r="D18" s="20"/>
+      <c r="E18" s="21"/>
+    </row>
+    <row r="19" spans="2:5">
+      <c r="B19" s="14">
+        <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="C19" s="15"/>
-      <c r="D19" s="16"/>
-      <c r="E19" s="16"/>
-    </row>
-    <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B20" s="6" t="n">
-        <f aca="false">B19+1</f>
+      <c r="C19" s="20"/>
+      <c r="D19" s="21"/>
+      <c r="E19" s="21"/>
+    </row>
+    <row r="20" spans="2:5">
+      <c r="B20" s="14">
+        <f t="shared" si="0"/>
         <v>11</v>
       </c>
-      <c r="C20" s="15"/>
-      <c r="D20" s="15"/>
-      <c r="E20" s="16"/>
-    </row>
-    <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B21" s="6" t="n">
-        <f aca="false">B20+1</f>
+      <c r="C20" s="20"/>
+      <c r="D20" s="20"/>
+      <c r="E20" s="21"/>
+    </row>
+    <row r="21" spans="2:5">
+      <c r="B21" s="14">
+        <f t="shared" si="0"/>
         <v>12</v>
       </c>
-      <c r="C21" s="15"/>
-      <c r="D21" s="15"/>
-      <c r="E21" s="16"/>
-    </row>
-    <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B22" s="6" t="n">
-        <f aca="false">B21+1</f>
+      <c r="C21" s="20"/>
+      <c r="D21" s="20"/>
+      <c r="E21" s="21"/>
+    </row>
+    <row r="22" spans="2:5">
+      <c r="B22" s="14">
+        <f t="shared" si="0"/>
         <v>13</v>
       </c>
-      <c r="C22" s="15"/>
-      <c r="D22" s="15"/>
-      <c r="E22" s="16"/>
-    </row>
-    <row r="23" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B23" s="6" t="n">
-        <f aca="false">B22+1</f>
+      <c r="C22" s="20"/>
+      <c r="D22" s="20"/>
+      <c r="E22" s="21"/>
+    </row>
+    <row r="23" spans="2:5">
+      <c r="B23" s="14">
+        <f t="shared" si="0"/>
         <v>14</v>
       </c>
-      <c r="C23" s="15"/>
-      <c r="D23" s="15"/>
-      <c r="E23" s="16"/>
-    </row>
-    <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B24" s="6" t="n">
-        <f aca="false">B23+1</f>
+      <c r="C23" s="20"/>
+      <c r="D23" s="20"/>
+      <c r="E23" s="21"/>
+    </row>
+    <row r="24" spans="2:5">
+      <c r="B24" s="14">
+        <f t="shared" si="0"/>
         <v>15</v>
       </c>
-      <c r="C24" s="15"/>
-      <c r="D24" s="15"/>
-      <c r="E24" s="16"/>
-    </row>
-    <row r="25" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B25" s="6" t="n">
-        <f aca="false">B24+1</f>
+      <c r="C24" s="20"/>
+      <c r="D24" s="20"/>
+      <c r="E24" s="21"/>
+    </row>
+    <row r="25" spans="2:5">
+      <c r="B25" s="14">
+        <f t="shared" si="0"/>
         <v>16</v>
       </c>
-      <c r="C25" s="15"/>
-      <c r="D25" s="15"/>
-      <c r="E25" s="16"/>
-    </row>
-    <row r="26" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B26" s="6" t="n">
-        <f aca="false">B25+1</f>
+      <c r="C25" s="20"/>
+      <c r="D25" s="20"/>
+      <c r="E25" s="21"/>
+    </row>
+    <row r="26" spans="2:5">
+      <c r="B26" s="14">
+        <f t="shared" si="0"/>
         <v>17</v>
       </c>
-      <c r="C26" s="15"/>
-      <c r="D26" s="15"/>
-      <c r="E26" s="16"/>
-    </row>
-    <row r="28" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C28" s="18" t="s">
+      <c r="C26" s="20"/>
+      <c r="D26" s="20"/>
+      <c r="E26" s="21"/>
+    </row>
+    <row r="28" spans="2:5">
+      <c r="C28" s="23" t="s">
         <v>29</v>
       </c>
-      <c r="D28" s="19"/>
-      <c r="E28" s="15"/>
+      <c r="D28" s="24"/>
+      <c r="E28" s="20"/>
     </row>
   </sheetData>
   <mergeCells count="6">
+    <mergeCell ref="D7:E7"/>
     <mergeCell ref="H1:J1"/>
     <mergeCell ref="B2:E2"/>
     <mergeCell ref="D4:E4"/>
     <mergeCell ref="D5:E5"/>
     <mergeCell ref="D6:E6"/>
-    <mergeCell ref="D7:E7"/>
   </mergeCells>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <sheetPr>
     <tabColor rgb="FF8EB4E3"/>
-    <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:J32"/>
-  <sheetFormatPr defaultColWidth="8.90234375" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:AMJ32"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="8.89"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="12.22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="16.22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="41.44"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="8" min="6" style="1" width="8.89"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="26.78"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1024" min="10" style="1" width="8.89"/>
+    <col min="1" max="1" width="8.88671875" style="11"/>
+    <col min="2" max="2" width="12.21875" style="11" customWidth="1"/>
+    <col min="3" max="3" width="16.21875" style="11" customWidth="1"/>
+    <col min="4" max="4" width="18" style="11" customWidth="1"/>
+    <col min="5" max="5" width="41.44140625" style="11" customWidth="1"/>
+    <col min="6" max="8" width="8.88671875" style="11"/>
+    <col min="9" max="9" width="26.77734375" style="11" customWidth="1"/>
+    <col min="10" max="1024" width="8.88671875" style="11"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2"/>
-      <c r="B1" s="3" t="s">
+    <row r="1" spans="1:10" ht="15.6">
+      <c r="A1" s="12"/>
+      <c r="B1" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="H1" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="I1" s="4"/>
-      <c r="J1" s="4"/>
-    </row>
-    <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B2" s="5" t="s">
+      <c r="I1" s="10"/>
+      <c r="J1" s="10"/>
+    </row>
+    <row r="2" spans="1:10">
+      <c r="B2" s="9" t="s">
         <v>41</v>
       </c>
-      <c r="C2" s="5"/>
-      <c r="D2" s="5"/>
-      <c r="E2" s="5"/>
-      <c r="H2" s="6"/>
-      <c r="I2" s="6" t="s">
+      <c r="C2" s="9"/>
+      <c r="D2" s="9"/>
+      <c r="E2" s="9"/>
+      <c r="H2" s="14"/>
+      <c r="I2" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="J2" s="6" t="s">
+      <c r="J2" s="14" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H3" s="6" t="s">
+    <row r="3" spans="1:10">
+      <c r="H3" s="14" t="s">
         <v>5</v>
       </c>
-      <c r="I3" s="6"/>
-      <c r="J3" s="6"/>
-    </row>
-    <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C4" s="23" t="s">
+      <c r="I3" s="14" t="s">
+        <v>6</v>
+      </c>
+      <c r="J3" s="14">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10">
+      <c r="C4" s="26" t="s">
         <v>7</v>
       </c>
-      <c r="D4" s="24" t="s">
+      <c r="D4" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="E4" s="24"/>
-      <c r="H4" s="6" t="s">
+      <c r="E4" s="3"/>
+      <c r="H4" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="I4" s="6"/>
-      <c r="J4" s="6"/>
-    </row>
-    <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C5" s="23" t="s">
+      <c r="I4" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="J4" s="14">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10">
+      <c r="C5" s="26" t="s">
         <v>11</v>
       </c>
-      <c r="D5" s="25" t="s">
+      <c r="D5" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="E5" s="25"/>
-      <c r="H5" s="6" t="s">
+      <c r="E5" s="2"/>
+      <c r="H5" s="14" t="s">
         <v>13</v>
       </c>
-      <c r="I5" s="6"/>
-      <c r="J5" s="6"/>
-    </row>
-    <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B6" s="10"/>
-      <c r="C6" s="11" t="s">
+      <c r="I5" s="14" t="s">
+        <v>14</v>
+      </c>
+      <c r="J5" s="14">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10">
+      <c r="B6" s="16"/>
+      <c r="C6" s="17" t="s">
         <v>15</v>
       </c>
-      <c r="D6" s="12"/>
-      <c r="E6" s="12"/>
-    </row>
-    <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C7" s="11" t="s">
+      <c r="D6" s="6"/>
+      <c r="E6" s="6"/>
+    </row>
+    <row r="7" spans="1:10">
+      <c r="C7" s="17" t="s">
         <v>16</v>
       </c>
-      <c r="D7" s="12"/>
-      <c r="E7" s="12"/>
-    </row>
-    <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B9" s="13" t="s">
+      <c r="D7" s="6"/>
+      <c r="E7" s="6"/>
+    </row>
+    <row r="9" spans="1:10">
+      <c r="B9" s="18" t="s">
         <v>18</v>
       </c>
-      <c r="C9" s="13" t="s">
+      <c r="C9" s="18" t="s">
         <v>19</v>
       </c>
-      <c r="D9" s="13" t="s">
+      <c r="D9" s="18" t="s">
         <v>20</v>
       </c>
-      <c r="E9" s="13" t="s">
+      <c r="E9" s="18" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B10" s="6" t="n">
+    <row r="10" spans="1:10">
+      <c r="B10" s="14">
         <v>1</v>
       </c>
-      <c r="C10" s="1" t="s">
+      <c r="C10" s="11" t="s">
         <v>44</v>
       </c>
-      <c r="D10" s="1" t="s">
+      <c r="D10" s="11" t="s">
         <v>45</v>
       </c>
-      <c r="E10" s="1" t="s">
+      <c r="E10" s="11" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="28.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B11" s="6" t="n">
-        <f aca="false">B10+1</f>
+    <row r="11" spans="1:10" ht="28.8">
+      <c r="B11" s="14">
+        <f t="shared" ref="B11:B30" si="0">B10+1</f>
         <v>2</v>
       </c>
-      <c r="C11" s="15" t="s">
+      <c r="C11" s="20" t="s">
         <v>47</v>
       </c>
-      <c r="D11" s="16" t="s">
+      <c r="D11" s="21" t="s">
         <v>48</v>
       </c>
-      <c r="E11" s="16" t="s">
+      <c r="E11" s="21" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="28.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B12" s="6" t="n">
-        <f aca="false">B11+1</f>
+    <row r="12" spans="1:10" ht="28.8">
+      <c r="B12" s="14">
+        <f t="shared" si="0"/>
         <v>3</v>
       </c>
-      <c r="C12" s="15" t="s">
+      <c r="C12" s="20" t="s">
         <v>44</v>
       </c>
-      <c r="D12" s="15" t="s">
+      <c r="D12" s="20" t="s">
         <v>50</v>
       </c>
-      <c r="E12" s="16" t="s">
+      <c r="E12" s="21" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B13" s="6" t="n">
-        <f aca="false">B12+1</f>
+    <row r="13" spans="1:10">
+      <c r="B13" s="14">
+        <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="C13" s="15"/>
-      <c r="D13" s="16"/>
-      <c r="E13" s="16"/>
-    </row>
-    <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B14" s="6" t="n">
-        <f aca="false">B13+1</f>
+      <c r="C13" s="20"/>
+      <c r="D13" s="21"/>
+      <c r="E13" s="21"/>
+    </row>
+    <row r="14" spans="1:10">
+      <c r="B14" s="14">
+        <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="C14" s="15"/>
-      <c r="D14" s="16"/>
-      <c r="E14" s="16"/>
-    </row>
-    <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B15" s="6" t="n">
-        <f aca="false">B14+1</f>
+      <c r="C14" s="20"/>
+      <c r="D14" s="21"/>
+      <c r="E14" s="21"/>
+    </row>
+    <row r="15" spans="1:10">
+      <c r="B15" s="14">
+        <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="C15" s="15"/>
-      <c r="D15" s="16"/>
-      <c r="E15" s="16"/>
-    </row>
-    <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B16" s="6" t="n">
-        <f aca="false">B15+1</f>
+      <c r="C15" s="20"/>
+      <c r="D15" s="21"/>
+      <c r="E15" s="21"/>
+    </row>
+    <row r="16" spans="1:10">
+      <c r="B16" s="14">
+        <f t="shared" si="0"/>
         <v>7</v>
       </c>
-      <c r="C16" s="15"/>
-      <c r="D16" s="16"/>
-      <c r="E16" s="16"/>
-    </row>
-    <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B17" s="6" t="n">
-        <f aca="false">B16+1</f>
+      <c r="C16" s="20"/>
+      <c r="D16" s="21"/>
+      <c r="E16" s="21"/>
+    </row>
+    <row r="17" spans="2:5">
+      <c r="B17" s="14">
+        <f t="shared" si="0"/>
         <v>8</v>
       </c>
-      <c r="C17" s="15"/>
-      <c r="D17" s="16"/>
-      <c r="E17" s="16"/>
-    </row>
-    <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B18" s="6" t="n">
-        <f aca="false">B17+1</f>
+      <c r="C17" s="20"/>
+      <c r="D17" s="21"/>
+      <c r="E17" s="21"/>
+    </row>
+    <row r="18" spans="2:5">
+      <c r="B18" s="14">
+        <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="C18" s="15"/>
-      <c r="D18" s="16"/>
-      <c r="E18" s="16"/>
-    </row>
-    <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B19" s="6" t="n">
-        <f aca="false">B18+1</f>
+      <c r="C18" s="20"/>
+      <c r="D18" s="21"/>
+      <c r="E18" s="21"/>
+    </row>
+    <row r="19" spans="2:5">
+      <c r="B19" s="14">
+        <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="C19" s="15"/>
-      <c r="D19" s="15"/>
-      <c r="E19" s="16"/>
-    </row>
-    <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B20" s="6" t="n">
-        <f aca="false">B19+1</f>
+      <c r="C19" s="20"/>
+      <c r="D19" s="20"/>
+      <c r="E19" s="21"/>
+    </row>
+    <row r="20" spans="2:5">
+      <c r="B20" s="14">
+        <f t="shared" si="0"/>
         <v>11</v>
       </c>
-      <c r="C20" s="15"/>
-      <c r="D20" s="16"/>
-      <c r="E20" s="16"/>
-    </row>
-    <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B21" s="6" t="n">
-        <f aca="false">B20+1</f>
+      <c r="C20" s="20"/>
+      <c r="D20" s="21"/>
+      <c r="E20" s="21"/>
+    </row>
+    <row r="21" spans="2:5">
+      <c r="B21" s="14">
+        <f t="shared" si="0"/>
         <v>12</v>
       </c>
-      <c r="C21" s="15"/>
-      <c r="D21" s="15"/>
-      <c r="E21" s="16"/>
-    </row>
-    <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B22" s="6" t="n">
-        <f aca="false">B21+1</f>
+      <c r="C21" s="20"/>
+      <c r="D21" s="20"/>
+      <c r="E21" s="21"/>
+    </row>
+    <row r="22" spans="2:5">
+      <c r="B22" s="14">
+        <f t="shared" si="0"/>
         <v>13</v>
       </c>
-      <c r="C22" s="15"/>
-      <c r="D22" s="16"/>
-      <c r="E22" s="16"/>
-    </row>
-    <row r="23" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B23" s="6" t="n">
-        <f aca="false">B22+1</f>
+      <c r="C22" s="20"/>
+      <c r="D22" s="21"/>
+      <c r="E22" s="21"/>
+    </row>
+    <row r="23" spans="2:5">
+      <c r="B23" s="14">
+        <f t="shared" si="0"/>
         <v>14</v>
       </c>
-      <c r="C23" s="15"/>
-      <c r="D23" s="16"/>
-      <c r="E23" s="16"/>
-    </row>
-    <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B24" s="6" t="n">
-        <f aca="false">B23+1</f>
+      <c r="C23" s="20"/>
+      <c r="D23" s="21"/>
+      <c r="E23" s="21"/>
+    </row>
+    <row r="24" spans="2:5">
+      <c r="B24" s="14">
+        <f t="shared" si="0"/>
         <v>15</v>
       </c>
-      <c r="C24" s="15"/>
-      <c r="D24" s="16"/>
-      <c r="E24" s="16"/>
-    </row>
-    <row r="25" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B25" s="6" t="n">
-        <f aca="false">B24+1</f>
+      <c r="C24" s="20"/>
+      <c r="D24" s="21"/>
+      <c r="E24" s="21"/>
+    </row>
+    <row r="25" spans="2:5">
+      <c r="B25" s="14">
+        <f t="shared" si="0"/>
         <v>16</v>
       </c>
-      <c r="C25" s="15"/>
-      <c r="D25" s="16"/>
-      <c r="E25" s="16"/>
-    </row>
-    <row r="26" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B26" s="6" t="n">
-        <f aca="false">B25+1</f>
+      <c r="C25" s="20"/>
+      <c r="D25" s="21"/>
+      <c r="E25" s="21"/>
+    </row>
+    <row r="26" spans="2:5">
+      <c r="B26" s="14">
+        <f t="shared" si="0"/>
         <v>17</v>
       </c>
-      <c r="C26" s="15"/>
-      <c r="D26" s="15"/>
-      <c r="E26" s="16"/>
-    </row>
-    <row r="27" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B27" s="6" t="n">
-        <f aca="false">B26+1</f>
+      <c r="C26" s="20"/>
+      <c r="D26" s="20"/>
+      <c r="E26" s="21"/>
+    </row>
+    <row r="27" spans="2:5">
+      <c r="B27" s="14">
+        <f t="shared" si="0"/>
         <v>18</v>
       </c>
-      <c r="C27" s="15"/>
-      <c r="D27" s="16"/>
-      <c r="E27" s="15"/>
-    </row>
-    <row r="28" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B28" s="6" t="n">
-        <f aca="false">B27+1</f>
+      <c r="C27" s="20"/>
+      <c r="D27" s="21"/>
+      <c r="E27" s="20"/>
+    </row>
+    <row r="28" spans="2:5">
+      <c r="B28" s="14">
+        <f t="shared" si="0"/>
         <v>19</v>
       </c>
-      <c r="C28" s="15"/>
-      <c r="D28" s="16"/>
-      <c r="E28" s="16"/>
-    </row>
-    <row r="29" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B29" s="6" t="n">
-        <f aca="false">B28+1</f>
+      <c r="C28" s="20"/>
+      <c r="D28" s="21"/>
+      <c r="E28" s="21"/>
+    </row>
+    <row r="29" spans="2:5">
+      <c r="B29" s="14">
+        <f t="shared" si="0"/>
         <v>20</v>
       </c>
-      <c r="C29" s="15"/>
-      <c r="D29" s="16"/>
-      <c r="E29" s="16"/>
-    </row>
-    <row r="30" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B30" s="6" t="n">
-        <f aca="false">B29+1</f>
+      <c r="C29" s="20"/>
+      <c r="D29" s="21"/>
+      <c r="E29" s="21"/>
+    </row>
+    <row r="30" spans="2:5">
+      <c r="B30" s="14">
+        <f t="shared" si="0"/>
         <v>21</v>
       </c>
-      <c r="C30" s="15"/>
-      <c r="D30" s="16"/>
-      <c r="E30" s="16"/>
-    </row>
-    <row r="32" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C32" s="18" t="s">
+      <c r="C30" s="20"/>
+      <c r="D30" s="21"/>
+      <c r="E30" s="21"/>
+    </row>
+    <row r="32" spans="2:5">
+      <c r="C32" s="23" t="s">
         <v>29</v>
       </c>
-      <c r="D32" s="19"/>
-      <c r="E32" s="15"/>
+      <c r="D32" s="24"/>
+      <c r="E32" s="20"/>
     </row>
   </sheetData>
   <mergeCells count="6">
+    <mergeCell ref="D7:E7"/>
     <mergeCell ref="H1:J1"/>
     <mergeCell ref="B2:E2"/>
     <mergeCell ref="D4:E4"/>
     <mergeCell ref="D5:E5"/>
     <mergeCell ref="D6:E6"/>
-    <mergeCell ref="D7:E7"/>
   </mergeCells>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+  <sheetPr>
     <tabColor rgb="FFEBF1DE"/>
-    <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:J32"/>
-  <sheetFormatPr defaultColWidth="8.90234375" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:AMJ32"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="8.89"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="12.22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="29.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="45.03"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="87.38"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="92.53"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="8" min="7" style="1" width="8.89"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="26.78"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1024" min="10" style="1" width="8.89"/>
+    <col min="1" max="1" width="8.88671875" style="11"/>
+    <col min="2" max="2" width="12.21875" style="11" customWidth="1"/>
+    <col min="3" max="3" width="29.6640625" style="11" customWidth="1"/>
+    <col min="4" max="4" width="45" style="11" customWidth="1"/>
+    <col min="5" max="5" width="87.33203125" style="11" customWidth="1"/>
+    <col min="6" max="6" width="92.5546875" style="11" customWidth="1"/>
+    <col min="7" max="8" width="8.88671875" style="11"/>
+    <col min="9" max="9" width="26.77734375" style="11" customWidth="1"/>
+    <col min="10" max="1024" width="8.88671875" style="11"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2"/>
-      <c r="B1" s="3" t="s">
+    <row r="1" spans="1:10" ht="15.6">
+      <c r="A1" s="12"/>
+      <c r="B1" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="H1" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="I1" s="4"/>
-      <c r="J1" s="4"/>
-    </row>
-    <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B2" s="5" t="s">
+      <c r="I1" s="10"/>
+      <c r="J1" s="10"/>
+    </row>
+    <row r="2" spans="1:10">
+      <c r="B2" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="C2" s="5"/>
-      <c r="D2" s="5"/>
-      <c r="E2" s="5"/>
-      <c r="H2" s="6"/>
-      <c r="I2" s="6" t="s">
+      <c r="C2" s="9"/>
+      <c r="D2" s="9"/>
+      <c r="E2" s="9"/>
+      <c r="H2" s="14"/>
+      <c r="I2" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="J2" s="6" t="s">
+      <c r="J2" s="14" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H3" s="6" t="s">
+    <row r="3" spans="1:10">
+      <c r="H3" s="14" t="s">
         <v>5</v>
       </c>
-      <c r="I3" s="6"/>
-      <c r="J3" s="6"/>
-    </row>
-    <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C4" s="23" t="s">
+      <c r="I3" s="14" t="s">
+        <v>6</v>
+      </c>
+      <c r="J3" s="14">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10">
+      <c r="C4" s="26" t="s">
         <v>53</v>
       </c>
-      <c r="D4" s="24" t="s">
+      <c r="D4" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="E4" s="24"/>
-      <c r="H4" s="6" t="s">
+      <c r="E4" s="3"/>
+      <c r="H4" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="I4" s="6"/>
-      <c r="J4" s="6"/>
-    </row>
-    <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C5" s="11" t="s">
+      <c r="I4" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="J4" s="14">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10">
+      <c r="C5" s="17" t="s">
         <v>15</v>
       </c>
-      <c r="D5" s="12" t="s">
+      <c r="D5" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="E5" s="12"/>
-      <c r="H5" s="6" t="s">
+      <c r="E5" s="6"/>
+      <c r="H5" s="14" t="s">
         <v>13</v>
       </c>
-      <c r="I5" s="6"/>
-      <c r="J5" s="6"/>
-    </row>
-    <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B6" s="10"/>
-      <c r="C6" s="11" t="s">
+      <c r="I5" s="14" t="s">
+        <v>14</v>
+      </c>
+      <c r="J5" s="14">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10">
+      <c r="B6" s="16"/>
+      <c r="C6" s="17" t="s">
         <v>16</v>
       </c>
-      <c r="D6" s="12" t="s">
+      <c r="D6" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="E6" s="12"/>
-    </row>
-    <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B9" s="13" t="s">
+      <c r="E6" s="6"/>
+    </row>
+    <row r="9" spans="1:10">
+      <c r="B9" s="18" t="s">
         <v>18</v>
       </c>
-      <c r="C9" s="13" t="s">
+      <c r="C9" s="18" t="s">
         <v>57</v>
       </c>
-      <c r="D9" s="13" t="s">
+      <c r="D9" s="18" t="s">
         <v>58</v>
       </c>
-      <c r="E9" s="13" t="s">
+      <c r="E9" s="18" t="s">
         <v>59</v>
       </c>
-      <c r="F9" s="13" t="s">
+      <c r="F9" s="18" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="202.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B10" s="6" t="n">
+    <row r="10" spans="1:10" ht="240">
+      <c r="B10" s="14">
         <v>1</v>
       </c>
-      <c r="C10" s="26" t="s">
+      <c r="C10" s="27" t="s">
         <v>61</v>
       </c>
-      <c r="D10" s="27" t="s">
+      <c r="D10" s="28" t="s">
         <v>62</v>
       </c>
-      <c r="E10" s="28" t="s">
+      <c r="E10" s="29" t="s">
         <v>63</v>
       </c>
-      <c r="F10" s="28" t="s">
+      <c r="F10" s="29" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="216.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B11" s="6" t="n">
-        <f aca="false">B10+1</f>
+    <row r="11" spans="1:10" ht="270">
+      <c r="B11" s="14">
+        <f t="shared" ref="B11:B30" si="0">B10+1</f>
         <v>2</v>
       </c>
-      <c r="C11" s="26" t="s">
+      <c r="C11" s="27" t="s">
         <v>65</v>
       </c>
-      <c r="D11" s="26" t="s">
+      <c r="D11" s="27" t="s">
         <v>62</v>
       </c>
-      <c r="E11" s="28" t="s">
+      <c r="E11" s="29" t="s">
         <v>66</v>
       </c>
-      <c r="F11" s="28" t="s">
+      <c r="F11" s="29" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="216.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B12" s="6" t="n">
-        <f aca="false">B11+1</f>
+    <row r="12" spans="1:10" ht="255">
+      <c r="B12" s="14">
+        <f t="shared" si="0"/>
         <v>3</v>
       </c>
-      <c r="C12" s="26" t="s">
+      <c r="C12" s="27" t="s">
         <v>68</v>
       </c>
-      <c r="D12" s="26" t="s">
+      <c r="D12" s="27" t="s">
         <v>62</v>
       </c>
-      <c r="E12" s="28" t="s">
+      <c r="E12" s="29" t="s">
         <v>69</v>
       </c>
-      <c r="F12" s="28" t="s">
+      <c r="F12" s="29" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B13" s="6" t="n">
-        <f aca="false">B12+1</f>
+    <row r="13" spans="1:10" ht="60">
+      <c r="B13" s="14">
+        <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="C13" s="26" t="s">
+      <c r="C13" s="27" t="s">
         <v>71</v>
       </c>
-      <c r="D13" s="27" t="s">
+      <c r="D13" s="28" t="s">
         <v>72</v>
       </c>
-      <c r="E13" s="28" t="s">
+      <c r="E13" s="29" t="s">
         <v>73</v>
       </c>
-      <c r="F13" s="28" t="s">
+      <c r="F13" s="29" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="108.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B14" s="6" t="n">
-        <f aca="false">B13+1</f>
+    <row r="14" spans="1:10" ht="135">
+      <c r="B14" s="14">
+        <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="C14" s="26" t="s">
+      <c r="C14" s="27" t="s">
         <v>75</v>
       </c>
-      <c r="D14" s="27" t="s">
+      <c r="D14" s="28" t="s">
         <v>76</v>
       </c>
-      <c r="E14" s="28" t="s">
+      <c r="E14" s="29" t="s">
         <v>77</v>
       </c>
-      <c r="F14" s="28" t="s">
+      <c r="F14" s="29" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B15" s="6" t="n">
-        <f aca="false">B14+1</f>
+    <row r="15" spans="1:10" ht="43.2">
+      <c r="B15" s="14">
+        <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="C15" s="26" t="s">
+      <c r="C15" s="27" t="s">
         <v>79</v>
       </c>
-      <c r="D15" s="27" t="s">
+      <c r="D15" s="28" t="s">
         <v>80</v>
       </c>
-      <c r="E15" s="29" t="s">
+      <c r="E15" s="30" t="s">
         <v>81</v>
       </c>
-      <c r="F15" s="30" t="s">
+      <c r="F15" s="31" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B16" s="6" t="n">
-        <f aca="false">B15+1</f>
+    <row r="16" spans="1:10" ht="28.8">
+      <c r="B16" s="14">
+        <f t="shared" si="0"/>
         <v>7</v>
       </c>
-      <c r="C16" s="26" t="s">
+      <c r="C16" s="27" t="s">
         <v>83</v>
       </c>
-      <c r="D16" s="27" t="s">
+      <c r="D16" s="28" t="s">
         <v>84</v>
       </c>
-      <c r="E16" s="29" t="s">
+      <c r="E16" s="30" t="s">
         <v>85</v>
       </c>
-      <c r="F16" s="16" t="s">
+      <c r="F16" s="21" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B17" s="6" t="n">
-        <f aca="false">B16+1</f>
+    <row r="17" spans="2:6">
+      <c r="B17" s="14">
+        <f t="shared" si="0"/>
         <v>8</v>
       </c>
-      <c r="C17" s="15"/>
-      <c r="D17" s="16"/>
-      <c r="E17" s="16"/>
-      <c r="F17" s="16"/>
-    </row>
-    <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B18" s="6" t="n">
-        <f aca="false">B17+1</f>
+      <c r="C17" s="20"/>
+      <c r="D17" s="21"/>
+      <c r="E17" s="21"/>
+      <c r="F17" s="21"/>
+    </row>
+    <row r="18" spans="2:6">
+      <c r="B18" s="14">
+        <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="C18" s="15"/>
-      <c r="D18" s="16"/>
-      <c r="E18" s="16"/>
-      <c r="F18" s="16"/>
-    </row>
-    <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B19" s="6" t="n">
-        <f aca="false">B18+1</f>
+      <c r="C18" s="20"/>
+      <c r="D18" s="21"/>
+      <c r="E18" s="21"/>
+      <c r="F18" s="21"/>
+    </row>
+    <row r="19" spans="2:6">
+      <c r="B19" s="14">
+        <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="C19" s="15"/>
-      <c r="D19" s="15"/>
-      <c r="E19" s="16"/>
-      <c r="F19" s="16"/>
-    </row>
-    <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B20" s="6" t="n">
-        <f aca="false">B19+1</f>
+      <c r="C19" s="20"/>
+      <c r="D19" s="20"/>
+      <c r="E19" s="21"/>
+      <c r="F19" s="21"/>
+    </row>
+    <row r="20" spans="2:6">
+      <c r="B20" s="14">
+        <f t="shared" si="0"/>
         <v>11</v>
       </c>
-      <c r="C20" s="15"/>
-      <c r="D20" s="16"/>
-      <c r="E20" s="16"/>
-      <c r="F20" s="16"/>
-    </row>
-    <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B21" s="6" t="n">
-        <f aca="false">B20+1</f>
+      <c r="C20" s="20"/>
+      <c r="D20" s="21"/>
+      <c r="E20" s="21"/>
+      <c r="F20" s="21"/>
+    </row>
+    <row r="21" spans="2:6">
+      <c r="B21" s="14">
+        <f t="shared" si="0"/>
         <v>12</v>
       </c>
-      <c r="C21" s="15"/>
-      <c r="D21" s="15"/>
-      <c r="E21" s="16"/>
-      <c r="F21" s="16"/>
-    </row>
-    <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B22" s="6" t="n">
-        <f aca="false">B21+1</f>
+      <c r="C21" s="20"/>
+      <c r="D21" s="20"/>
+      <c r="E21" s="21"/>
+      <c r="F21" s="21"/>
+    </row>
+    <row r="22" spans="2:6">
+      <c r="B22" s="14">
+        <f t="shared" si="0"/>
         <v>13</v>
       </c>
-      <c r="C22" s="15"/>
-      <c r="D22" s="16"/>
-      <c r="E22" s="16"/>
-      <c r="F22" s="16"/>
-    </row>
-    <row r="23" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B23" s="6" t="n">
-        <f aca="false">B22+1</f>
+      <c r="C22" s="20"/>
+      <c r="D22" s="21"/>
+      <c r="E22" s="21"/>
+      <c r="F22" s="21"/>
+    </row>
+    <row r="23" spans="2:6">
+      <c r="B23" s="14">
+        <f t="shared" si="0"/>
         <v>14</v>
       </c>
-      <c r="C23" s="15"/>
-      <c r="D23" s="16"/>
-      <c r="E23" s="16"/>
-      <c r="F23" s="16"/>
-    </row>
-    <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B24" s="6" t="n">
-        <f aca="false">B23+1</f>
+      <c r="C23" s="20"/>
+      <c r="D23" s="21"/>
+      <c r="E23" s="21"/>
+      <c r="F23" s="21"/>
+    </row>
+    <row r="24" spans="2:6">
+      <c r="B24" s="14">
+        <f t="shared" si="0"/>
         <v>15</v>
       </c>
-      <c r="C24" s="15"/>
-      <c r="D24" s="16"/>
-      <c r="E24" s="16"/>
-      <c r="F24" s="16"/>
-    </row>
-    <row r="25" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B25" s="6" t="n">
-        <f aca="false">B24+1</f>
+      <c r="C24" s="20"/>
+      <c r="D24" s="21"/>
+      <c r="E24" s="21"/>
+      <c r="F24" s="21"/>
+    </row>
+    <row r="25" spans="2:6">
+      <c r="B25" s="14">
+        <f t="shared" si="0"/>
         <v>16</v>
       </c>
-      <c r="C25" s="15"/>
-      <c r="D25" s="16"/>
-      <c r="E25" s="16"/>
-      <c r="F25" s="16"/>
-    </row>
-    <row r="26" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B26" s="6" t="n">
-        <f aca="false">B25+1</f>
+      <c r="C25" s="20"/>
+      <c r="D25" s="21"/>
+      <c r="E25" s="21"/>
+      <c r="F25" s="21"/>
+    </row>
+    <row r="26" spans="2:6">
+      <c r="B26" s="14">
+        <f t="shared" si="0"/>
         <v>17</v>
       </c>
-      <c r="C26" s="15"/>
-      <c r="D26" s="15"/>
-      <c r="E26" s="16"/>
-      <c r="F26" s="16"/>
-    </row>
-    <row r="27" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B27" s="6" t="n">
-        <f aca="false">B26+1</f>
+      <c r="C26" s="20"/>
+      <c r="D26" s="20"/>
+      <c r="E26" s="21"/>
+      <c r="F26" s="21"/>
+    </row>
+    <row r="27" spans="2:6">
+      <c r="B27" s="14">
+        <f t="shared" si="0"/>
         <v>18</v>
       </c>
-      <c r="C27" s="15"/>
-      <c r="D27" s="16"/>
-      <c r="E27" s="15"/>
-      <c r="F27" s="15"/>
-    </row>
-    <row r="28" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B28" s="6" t="n">
-        <f aca="false">B27+1</f>
+      <c r="C27" s="20"/>
+      <c r="D27" s="21"/>
+      <c r="E27" s="20"/>
+      <c r="F27" s="20"/>
+    </row>
+    <row r="28" spans="2:6">
+      <c r="B28" s="14">
+        <f t="shared" si="0"/>
         <v>19</v>
       </c>
-      <c r="C28" s="15"/>
-      <c r="D28" s="16"/>
-      <c r="E28" s="16"/>
-      <c r="F28" s="16"/>
-    </row>
-    <row r="29" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B29" s="6" t="n">
-        <f aca="false">B28+1</f>
+      <c r="C28" s="20"/>
+      <c r="D28" s="21"/>
+      <c r="E28" s="21"/>
+      <c r="F28" s="21"/>
+    </row>
+    <row r="29" spans="2:6">
+      <c r="B29" s="14">
+        <f t="shared" si="0"/>
         <v>20</v>
       </c>
-      <c r="C29" s="15"/>
-      <c r="D29" s="16"/>
-      <c r="E29" s="16"/>
-      <c r="F29" s="16"/>
-    </row>
-    <row r="30" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B30" s="6" t="n">
-        <f aca="false">B29+1</f>
+      <c r="C29" s="20"/>
+      <c r="D29" s="21"/>
+      <c r="E29" s="21"/>
+      <c r="F29" s="21"/>
+    </row>
+    <row r="30" spans="2:6">
+      <c r="B30" s="14">
+        <f t="shared" si="0"/>
         <v>21</v>
       </c>
-      <c r="C30" s="15"/>
-      <c r="D30" s="16"/>
-      <c r="E30" s="16"/>
-      <c r="F30" s="16"/>
-    </row>
-    <row r="32" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C32" s="31" t="s">
+      <c r="C30" s="20"/>
+      <c r="D30" s="21"/>
+      <c r="E30" s="21"/>
+      <c r="F30" s="21"/>
+    </row>
+    <row r="32" spans="2:6">
+      <c r="C32" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="D32" s="31"/>
-      <c r="E32" s="31"/>
+      <c r="D32" s="1"/>
+      <c r="E32" s="1"/>
       <c r="F32" s="32"/>
     </row>
   </sheetData>
   <mergeCells count="6">
+    <mergeCell ref="C32:E32"/>
     <mergeCell ref="H1:J1"/>
     <mergeCell ref="B2:E2"/>
     <mergeCell ref="D4:E4"/>
     <mergeCell ref="D5:E5"/>
     <mergeCell ref="D6:E6"/>
-    <mergeCell ref="C32:E32"/>
   </mergeCells>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
</xml_diff>